<commit_message>
Weekly SHOCAPP data 2026-03-13
</commit_message>
<xml_diff>
--- a/output/shocapp_report.xlsx
+++ b/output/shocapp_report.xlsx
@@ -889,6 +889,9 @@
       <c r="G22" t="str">
         <v>MIRTILLO</v>
       </c>
+      <c r="H22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1020,9 +1023,6 @@
       <c r="C29" t="str">
         <v>PISTACCHI</v>
       </c>
-      <c r="D29">
-        <v>3</v>
-      </c>
       <c r="E29" t="str">
         <v>PICCHIE</v>
       </c>
@@ -1030,7 +1030,7 @@
         <v>PERA GORGONZOLA</v>
       </c>
       <c r="H29">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1071,9 +1071,6 @@
       <c r="A32" t="str">
         <v>STRIA</v>
       </c>
-      <c r="B32">
-        <v>3</v>
-      </c>
       <c r="E32" t="str">
         <v>COPP. GRANDI</v>
       </c>
@@ -1100,7 +1097,7 @@
         <v>ZUCCA E SEMI</v>
       </c>
       <c r="H34">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add order-only PDF output and include it in Telegram bot
</commit_message>
<xml_diff>
--- a/output/shocapp_report.xlsx
+++ b/output/shocapp_report.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Ordini Settimanali 13-03-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Ordini Settimanali 15-03-2026" sheetId="1" r:id="rId1"/>
     <sheet name="Mantenimento" sheetId="2" r:id="rId2"/>
     <sheet name="Esaurito" sheetId="3" r:id="rId3"/>
     <sheet name="Da Ordinare" sheetId="4" r:id="rId4"/>
@@ -400,46 +400,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Flavor 1</v>
+        <v>Gelato</v>
       </c>
       <c r="B1" t="str">
-        <v>Qty 1</v>
+        <v>ORDINE</v>
       </c>
       <c r="C1" t="str">
-        <v>Flavor 2</v>
+        <v>Creme</v>
       </c>
       <c r="D1" t="str">
-        <v>Qty 2</v>
+        <v>ORDINE</v>
       </c>
       <c r="E1" t="str">
-        <v>Flavor 3</v>
+        <v>Cioccolati</v>
       </c>
       <c r="F1" t="str">
-        <v>Qty 3</v>
+        <v>ORDINE</v>
       </c>
       <c r="G1" t="str">
-        <v>Flavor 4</v>
+        <v>Sorbetti</v>
       </c>
       <c r="H1" t="str">
-        <v>Qty 4</v>
+        <v>ORDINE</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ARACHIDI</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
       <c r="C2" t="str">
-        <v>CREMA</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="E2" t="str">
         <v>CIOCCOLATO</v>
@@ -459,16 +456,16 @@
         <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C3" t="str">
-        <v>C. VANIGLIA</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3" t="str">
-        <v>C. LATTE</v>
+        <v>CIOCCOLATO AL LATTE GELATO</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -482,71 +479,68 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BAKLAVA</v>
+        <v>BASILICO NOCI E MIELE</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
       </c>
       <c r="C4" t="str">
-        <v>C. FRAGOLE</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E4" t="str">
-        <v>C. KENTUCKY</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="str">
-        <v>AMARENA E BIRRA</v>
+        <v>ANANAS E ZENZERO</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BASILICO NOCI E MELE</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C5" t="str">
-        <v>C. ZENZERO</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E5" t="str">
-        <v>C. MADAGASCAR</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
+        <v>CIOCCOLATO AL WHISKY</v>
       </c>
       <c r="G5" t="str">
-        <v>ANANAS E ZENZ.</v>
+        <v>ANGURIA</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BIANCANEVE</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="C6" t="str">
-        <v>C. CANNELLA</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6" t="str">
-        <v>C. VENEZUELA</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
+        <v>CIOCCOLATO BIANCO</v>
       </c>
       <c r="G6" t="str">
-        <v>ANGURIA</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -554,25 +548,25 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>CAFFÈ</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C7" t="str">
-        <v>C. AGNESE</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="D7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E7" t="str">
-        <v>C. PIMENTO</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="str">
-        <v>AVOCADO E LIME</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -580,85 +574,82 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CIOCC. BIANCO</v>
+        <v>COCCO CREMA</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
       </c>
       <c r="C8" t="str">
-        <v>C. LEMON CURD</v>
+        <v>CREMA PASTICCIERA PARISI</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>C. LAPSANG</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8" t="str">
-        <v>BANANA E LIME</v>
+        <v>CACHI</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>COCCO CREMA</v>
-      </c>
-      <c r="B9">
-        <v>2</v>
+        <v>CREMA BANANA E CROCCANTE AL SESAMO</v>
       </c>
       <c r="C9" t="str">
-        <v>CHEESE MIRT</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="D9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E9" t="str">
-        <v>C. WASABY</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
+        <v>CIOCCOLATO EQUADOR</v>
       </c>
       <c r="G9" t="str">
-        <v>CACHI</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
+        <v>CILIEGIA</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>C. BANANA</v>
-      </c>
-      <c r="B10">
-        <v>2</v>
+        <v>FICHI ALLA GRECA</v>
       </c>
       <c r="C10" t="str">
-        <v>CARROT LAKE</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
       </c>
       <c r="E10" t="str">
-        <v>C. ROSEMARY</v>
+        <v>CIOCCOLATO KENTUCKY</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
       </c>
       <c r="G10" t="str">
-        <v>CASTAGNA</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
+        <v>COCCO</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>FINOCCHIO</v>
+        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
       </c>
       <c r="C11" t="str">
-        <v>TIRAMISU</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11" t="str">
-        <v>C. PORCELLANA</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
       </c>
       <c r="G11" t="str">
         <v>COCCO AL RUM</v>
@@ -678,110 +669,101 @@
         <v>2</v>
       </c>
       <c r="E12" t="str">
-        <v>C. AMBOA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
       </c>
       <c r="G12" t="str">
-        <v>FICHI</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
       </c>
       <c r="C13" t="str">
-        <v>ZABAIONE</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="str">
-        <v>GIANDUIA</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="G13" t="str">
-        <v>FRAGOLA</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
+        <v>DRACARYS (dragon fruit, fragole &amp; peperoncino)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MENTA CIOCC.</v>
-      </c>
-      <c r="B14">
-        <v>2</v>
+        <v>LATTE &amp; CEREALI</v>
       </c>
       <c r="C14" t="str">
-        <v>Z. MOSCATO</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14" t="str">
-        <v>C. ARANCIA</v>
-      </c>
-      <c r="F14">
-        <v>1</v>
+        <v>CIOCCOLATO UGANDA</v>
       </c>
       <c r="G14" t="str">
-        <v>FRAG. CALVADOS</v>
+        <v>FEIJOA</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>M. BIANCA</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Z. RATAFIA</v>
+        <v>LATTE DI FICO (PAMPANELLA)</v>
       </c>
       <c r="E15" t="str">
-        <v>C. FRUTTOSIO</v>
+        <v>CIOCCOLATO VENEZUELA</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
       </c>
       <c r="G15" t="str">
-        <v>FRUTTI BOSCO</v>
-      </c>
-      <c r="H15">
-        <v>3</v>
+        <v>FICHI</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>M. TOSTATA</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
       </c>
       <c r="C16" t="str">
-        <v>Z. FATA</v>
+        <v>speciali</v>
       </c>
       <c r="E16" t="str">
-        <v>C. ESTASY</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16" t="str">
-        <v>LAMPONE</v>
-      </c>
-      <c r="H16">
-        <v>2</v>
+        <v>FICHI D INDIA</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>M. ARANCIA</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
       <c r="C17" t="str">
-        <v>Z. ZIBIBBO</v>
+        <v>ANGURIA, GIN, ZUCCHERO DI CANNA &amp; SALE MALDON</v>
       </c>
       <c r="E17" t="str">
-        <v>N. FRUTTOSIO</v>
+        <v>ESTASI</v>
       </c>
       <c r="G17" t="str">
-        <v>LIMONE</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -789,125 +771,110 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>M. CARDAMOMO</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C18" t="str">
-        <v>SACHER</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
+        <v>CASTAGNACCIO</v>
       </c>
       <c r="E18" t="str">
-        <v>V. GIANDUIA</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="G18" t="str">
-        <v>MANDARINO</v>
+        <v>FRAGOLE DI TERRACINA &amp; CHAMPAGNE</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>NOCCIOLA</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" t="str">
-        <v>NOCCIOLATA</v>
+        <v>COTOGNATA</v>
       </c>
       <c r="E19" t="str">
-        <v>P. VEGAN</v>
-      </c>
-      <c r="F19">
-        <v>1</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="G19" t="str">
-        <v>MANGO</v>
-      </c>
-      <c r="H19">
-        <v>0</v>
+        <v>FRAGOLINE DI BOSCO AL CALVADOS</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>NOCI E UVETTA</v>
+        <v>MANDORLA E ARANCIA</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
       </c>
       <c r="C20" t="str">
-        <v>LA-LA-</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
+        <v>CREMA COGNAC E NOCE MOSCATA</v>
       </c>
       <c r="E20" t="str">
-        <v>COPPA</v>
+        <v>GIANDUIA VARIEGATA</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
       </c>
       <c r="G20" t="str">
-        <v>MELA N. E C.</v>
-      </c>
-      <c r="H20">
-        <v>2</v>
+        <v>FRUTTI DI BOSCO (LAMPONE, RIBES, MORA, MIRTILLO)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>PERE BH</v>
-      </c>
-      <c r="B21">
-        <v>0</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="C21" t="str">
-        <v>STRACCHINO</v>
-      </c>
-      <c r="D21">
-        <v>1</v>
+        <v>CREMA DI FICHI SETTEMBRINI &amp; GRUE' DI LAMPONI</v>
       </c>
       <c r="E21" t="str">
-        <v>CIALDINE</v>
+        <v>MOU LATTE SALATO</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
       </c>
       <c r="G21" t="str">
-        <v>MELONE</v>
+        <v>HIBISCUS</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>POLLICINA</v>
+        <v>MONTBLANC</v>
       </c>
       <c r="B22">
         <v>2</v>
       </c>
       <c r="C22" t="str">
-        <v>LAVANDA</v>
-      </c>
-      <c r="D22">
-        <v>2</v>
+        <v>CREMA ELISIR BORSCI &amp; PINOLI TOSTATI</v>
       </c>
       <c r="E22" t="str">
-        <v>SUSHI GELATO</v>
+        <v>SACHER TORTE</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
       </c>
       <c r="G22" t="str">
-        <v>MIRTILLO</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="H22">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>BRONTE</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B23">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C23" t="str">
-        <v>NOCE BURRO</v>
-      </c>
-      <c r="E23" t="str">
-        <v>SUSHI TIRAMISU</v>
+        <v>FIORI DI MAGNOLIA &amp; LIME</v>
       </c>
       <c r="G23" t="str">
-        <v>MORA</v>
+        <v>LIMONE</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -915,36 +882,30 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>RICOTTA AGRUMI</v>
-      </c>
-      <c r="B24">
-        <v>1</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="C24" t="str">
-        <v>FIORDIFIOR</v>
+        <v>GELATO DI PANETTONE</v>
       </c>
       <c r="E24" t="str">
-        <v>SUSHI MISTI</v>
+        <v>Varie</v>
       </c>
       <c r="G24" t="str">
-        <v>PANACEA</v>
-      </c>
-      <c r="H24">
-        <v>1</v>
+        <v>MANDARINO</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>RICOTTA COCCO</v>
+        <v>NOCI E UVETTA DI CORINTO</v>
       </c>
       <c r="C25" t="str">
-        <v>PAMPANELLA</v>
+        <v>GELSI BIANCHI, SAKE' E ANACARDI SALATI</v>
       </c>
       <c r="E25" t="str">
-        <v>T.S. 6P</v>
+        <v>CAPRESE</v>
       </c>
       <c r="G25" t="str">
-        <v>PASSION</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -952,165 +913,358 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>RISO E VANIGLIA</v>
-      </c>
-      <c r="B26">
-        <v>1</v>
+        <v>NOCI PECAN</v>
       </c>
       <c r="C26" t="str">
-        <v>TORRONE</v>
+        <v>GORGONZOLA</v>
       </c>
       <c r="E26" t="str">
-        <v>T.S. 8P</v>
+        <v>CHICCHIAINI</v>
       </c>
       <c r="G26" t="str">
-        <v>PAPAYA</v>
+        <v>MELA MANDORLA E CANNELLA</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>STRACCIATELLA</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B27">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C27" t="str">
-        <v>PANETTONE</v>
-      </c>
-      <c r="D27">
-        <v>0</v>
+        <v>MATCHA-BASILICO-AVOCADO &amp; PERLE DI FRUTTA</v>
       </c>
       <c r="E27" t="str">
-        <v>T.G. 6P</v>
+        <v>CIALDINE</v>
       </c>
       <c r="G27" t="str">
-        <v>PENSIERO</v>
-      </c>
-      <c r="H27">
-        <v>0</v>
+        <v>MELOGRANO WONDERFUL</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SEADAS</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C28" t="str">
-        <v>MONTBLANC</v>
-      </c>
-      <c r="D28">
-        <v>1</v>
+        <v>MATE-LATE</v>
       </c>
       <c r="E28" t="str">
-        <v>T.G. 8P</v>
+        <v>CIOCCOLATA CALDA</v>
       </c>
       <c r="G28" t="str">
-        <v>PERA</v>
-      </c>
-      <c r="H28">
-        <v>0</v>
+        <v>MELONE</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>YOGURT</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C29" t="str">
-        <v>PISTACCHI</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="E29" t="str">
-        <v>PICCHIE</v>
+        <v>COPPA IN CIALDA</v>
       </c>
       <c r="G29" t="str">
-        <v>PERA GORGONZOLA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>VENERE</v>
+        <v>POLLICINA</v>
+      </c>
+      <c r="B30">
+        <v>0</v>
       </c>
       <c r="C30" t="str">
-        <v>RICE COCCO</v>
+        <v>NON TI SCORDAR DI ME</v>
       </c>
       <c r="E30" t="str">
-        <v>HUMA</v>
+        <v>COPPETTA GRANDE</v>
       </c>
       <c r="G30" t="str">
-        <v>PESCA AL VINO</v>
+        <v>MORA</v>
       </c>
       <c r="H30">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>THE VERDE</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31" t="str">
-        <v>LIM/MAS</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="E31" t="str">
-        <v>COPP. PICCOLE</v>
+        <v>COPPETTA PICCOLA</v>
       </c>
       <c r="G31" t="str">
-        <v>PUNCH</v>
+        <v>PANACEA (LATTE DI MANDORLA MENTA &amp; GINSENG)</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>STRIA</v>
+        <v>RICOTTA E FICHI ALLA GRECA</v>
+      </c>
+      <c r="C32" t="str">
+        <v>PECORINO</v>
       </c>
       <c r="E32" t="str">
-        <v>COPP. GRANDI</v>
+        <v>MOUSSE</v>
       </c>
       <c r="G32" t="str">
-        <v>UVA NOCI</v>
+        <v>PAPAYA</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
+      <c r="A33" t="str">
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33" t="str">
+        <v>PERA AL GORGONZOLA</v>
+      </c>
       <c r="E33" t="str">
-        <v>CAPRESE</v>
+        <v>SUSHI GELATO</v>
       </c>
       <c r="G33" t="str">
-        <v>UVA FRAGOLA</v>
+        <v>PASSION FRUIT</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
+      <c r="A34" t="str">
+        <v>RICOTTA, AMARENE &amp; NOCCIOLE PRALINATE</v>
+      </c>
+      <c r="C34" t="str">
+        <v>PERA E PECORINO DOP</v>
+      </c>
       <c r="E34" t="str">
-        <v>C. CALDA</v>
-      </c>
-      <c r="F34">
-        <v>2</v>
+        <v>SUSHI MISTI</v>
       </c>
       <c r="G34" t="str">
-        <v>ZUCCA E SEMI</v>
+        <v>PENSIERO</v>
       </c>
       <c r="H34">
         <v>0</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>RICOTTA, MIELE E COCCO</v>
+      </c>
+      <c r="C35" t="str">
+        <v>PESCA BIANCA AL BASILICO</v>
+      </c>
+      <c r="E35" t="str">
+        <v>SUSHI TIRAMISU</v>
+      </c>
+      <c r="G35" t="str">
+        <v>PERA</v>
+      </c>
+      <c r="H35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>RISO E VANIGLIA</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" t="str">
+        <v>PESCA TABACCHIERA</v>
+      </c>
+      <c r="E36" t="str">
+        <v>TORTA AGNESE 6P</v>
+      </c>
+      <c r="G36" t="str">
+        <v>PESCHE AL VINO</v>
+      </c>
+      <c r="H36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>SEADAS</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37" t="str">
+        <v>POMODORO DATTERINO</v>
+      </c>
+      <c r="E37" t="str">
+        <v>TORTA AGNESE 8P</v>
+      </c>
+      <c r="G37" t="str">
+        <v>PRUGNA ROSSA, FIORI D'IBISCO</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
+      </c>
+      <c r="C38" t="str">
+        <v>RISO AL COCCO &amp; SALSA AL MANGO PICCANTE</v>
+      </c>
+      <c r="E38" t="str">
+        <v>TORTA CHEESCAKE 6P</v>
+      </c>
+      <c r="G38" t="str">
+        <v>PRUGNE AL SAKE'</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="str">
+        <v>ROSA KAEKADE E ARANCIA</v>
+      </c>
+      <c r="E39" t="str">
+        <v>TORTA CHEESCAKE 8P</v>
+      </c>
+      <c r="G39" t="str">
+        <v>PUNCH PARADISE</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>STRACCIATELLA</v>
+      </c>
+      <c r="B40">
+        <v>4</v>
+      </c>
+      <c r="C40" t="str">
+        <v>STRACCIATELLA AL FIOR DI RISO</v>
+      </c>
+      <c r="E40" t="str">
+        <v>TORTA LAURA 6P</v>
+      </c>
+      <c r="G40" t="str">
+        <v>RIBES NERO</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TE VERDE MATCHA</v>
+      </c>
+      <c r="B41">
+        <v>0</v>
+      </c>
+      <c r="C41" t="str">
+        <v>TORRONE SALATO</v>
+      </c>
+      <c r="E41" t="str">
+        <v>TORTA LAURA 8P</v>
+      </c>
+      <c r="G41" t="str">
+        <v>UVA E NOCI</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>VENERE ROSA</v>
+      </c>
+      <c r="C42" t="str">
+        <v>VIRGIN BANANA (BANANA, COCCO LIMONE)</v>
+      </c>
+      <c r="E42" t="str">
+        <v>TORTA TIRAMISU 6P</v>
+      </c>
+      <c r="G42" t="str">
+        <v>UVA FRAGOLA E ZENZERO</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>YOGURT</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="str">
+        <v>ZABAIONE VIN SANTO OCCHIO DI PERNICE</v>
+      </c>
+      <c r="E43" t="str">
+        <v>TORTA TIRAMISU 8P</v>
+      </c>
+      <c r="G43" t="str">
+        <v>V. BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="G44" t="str">
+        <v>V. CASTAGNA AL WHISKY</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="G45" t="str">
+        <v>V. CASTAGNA E MIRTO</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="G46" t="str">
+        <v>V. EVERGREEN BRONTE VEGAN</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="G47" t="str">
+        <v>V. NOCCIOLA AL FRUTTOSIO</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="G48" t="str">
+        <v>ZUCCA COI SUOI SEMI CARAMELLATI</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H48"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1177,7 +1331,7 @@
         <v>Stock</v>
       </c>
       <c r="B4" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -1186,10 +1340,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E4" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="str">
-        <v>6.087</v>
+        <v>3.277</v>
       </c>
     </row>
     <row r="5">
@@ -1197,7 +1351,7 @@
         <v>Stock</v>
       </c>
       <c r="B5" t="str">
-        <v>BANANA E LIME</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="C5" t="str">
         <v/>
@@ -1206,10 +1360,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E5" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="str">
-        <v>2.466</v>
+        <v>9.098</v>
       </c>
     </row>
     <row r="6">
@@ -1217,7 +1371,7 @@
         <v>Stock</v>
       </c>
       <c r="B6" t="str">
-        <v>CACHI</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -1229,7 +1383,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="str">
-        <v>2.022</v>
+        <v>2.466</v>
       </c>
     </row>
     <row r="7">
@@ -1237,7 +1391,7 @@
         <v>Stock</v>
       </c>
       <c r="B7" t="str">
-        <v>CIOCCOLATO</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="C7" t="str">
         <v/>
@@ -1246,10 +1400,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E7" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F7" t="str">
-        <v>11.858</v>
+        <v>5.509</v>
       </c>
     </row>
     <row r="8">
@@ -1257,7 +1411,7 @@
         <v>Stock</v>
       </c>
       <c r="B8" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -1266,10 +1420,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E8" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="str">
-        <v>2.947</v>
+        <v>5.462</v>
       </c>
     </row>
     <row r="9">
@@ -1277,7 +1431,7 @@
         <v>Stock</v>
       </c>
       <c r="B9" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>CAFFE'</v>
       </c>
       <c r="C9" t="str">
         <v/>
@@ -1286,10 +1440,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E9" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" t="str">
-        <v>2.876</v>
+        <v>5.537</v>
       </c>
     </row>
     <row r="10">
@@ -1297,7 +1451,7 @@
         <v>Stock</v>
       </c>
       <c r="B10" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CACHI</v>
       </c>
       <c r="C10" t="str">
         <v/>
@@ -1309,7 +1463,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="str">
-        <v>3.057</v>
+        <v>2.022</v>
       </c>
     </row>
     <row r="11">
@@ -1317,7 +1471,7 @@
         <v>Stock</v>
       </c>
       <c r="B11" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="C11" t="str">
         <v/>
@@ -1326,10 +1480,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E11" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11" t="str">
-        <v>3.000</v>
+        <v>8.885</v>
       </c>
     </row>
     <row r="12">
@@ -1337,7 +1491,7 @@
         <v>Stock</v>
       </c>
       <c r="B12" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="C12" t="str">
         <v/>
@@ -1349,7 +1503,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="str">
-        <v>2.775</v>
+        <v>2.947</v>
       </c>
     </row>
     <row r="13">
@@ -1357,7 +1511,7 @@
         <v>Stock</v>
       </c>
       <c r="B13" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="C13" t="str">
         <v/>
@@ -1369,7 +1523,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="str">
-        <v>3.001</v>
+        <v>2.876</v>
       </c>
     </row>
     <row r="14">
@@ -1377,7 +1531,7 @@
         <v>Stock</v>
       </c>
       <c r="B14" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="C14" t="str">
         <v/>
@@ -1389,7 +1543,7 @@
         <v>1</v>
       </c>
       <c r="F14" t="str">
-        <v>2.881</v>
+        <v>3.057</v>
       </c>
     </row>
     <row r="15">
@@ -1397,7 +1551,7 @@
         <v>Stock</v>
       </c>
       <c r="B15" t="str">
-        <v>COCCO CREMA</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -1409,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="str">
-        <v>2.970</v>
+        <v>3.000</v>
       </c>
     </row>
     <row r="16">
@@ -1417,7 +1571,7 @@
         <v>Stock</v>
       </c>
       <c r="B16" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="C16" t="str">
         <v/>
@@ -1426,10 +1580,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E16" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="str">
-        <v>5.432</v>
+        <v>2.775</v>
       </c>
     </row>
     <row r="17">
@@ -1437,7 +1591,7 @@
         <v>Stock</v>
       </c>
       <c r="B17" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="C17" t="str">
         <v/>
@@ -1449,7 +1603,7 @@
         <v>1</v>
       </c>
       <c r="F17" t="str">
-        <v>2.616</v>
+        <v>3.001</v>
       </c>
     </row>
     <row r="18">
@@ -1457,7 +1611,7 @@
         <v>Stock</v>
       </c>
       <c r="B18" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="C18" t="str">
         <v/>
@@ -1469,7 +1623,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="str">
-        <v>2.819</v>
+        <v>2.881</v>
       </c>
     </row>
     <row r="19">
@@ -1477,7 +1631,7 @@
         <v>Stock</v>
       </c>
       <c r="B19" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="C19" t="str">
         <v/>
@@ -1489,7 +1643,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="str">
-        <v>2.708</v>
+        <v>2.970</v>
       </c>
     </row>
     <row r="20">
@@ -1497,7 +1651,7 @@
         <v>Stock</v>
       </c>
       <c r="B20" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="C20" t="str">
         <v/>
@@ -1506,10 +1660,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E20" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20" t="str">
-        <v>2.764</v>
+        <v>7.933</v>
       </c>
     </row>
     <row r="21">
@@ -1517,7 +1671,7 @@
         <v>Stock</v>
       </c>
       <c r="B21" t="str">
-        <v>FIORDILATTE</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="C21" t="str">
         <v/>
@@ -1526,10 +1680,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E21" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="str">
-        <v>5.909</v>
+        <v>2.527</v>
       </c>
     </row>
     <row r="22">
@@ -1537,7 +1691,7 @@
         <v>Stock</v>
       </c>
       <c r="B22" t="str">
-        <v>FRAGOLA</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="C22" t="str">
         <v/>
@@ -1546,10 +1700,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E22" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F22" t="str">
-        <v>9.486</v>
+        <v>2.616</v>
       </c>
     </row>
     <row r="23">
@@ -1557,7 +1711,7 @@
         <v>Stock</v>
       </c>
       <c r="B23" t="str">
-        <v>LEMON CURD</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="C23" t="str">
         <v/>
@@ -1569,7 +1723,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="str">
-        <v>2.609</v>
+        <v>2.819</v>
       </c>
     </row>
     <row r="24">
@@ -1577,7 +1731,7 @@
         <v>Stock</v>
       </c>
       <c r="B24" t="str">
-        <v>LIMONE</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="C24" t="str">
         <v/>
@@ -1586,10 +1740,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E24" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F24" t="str">
-        <v>10.105</v>
+        <v>2.708</v>
       </c>
     </row>
     <row r="25">
@@ -1597,7 +1751,7 @@
         <v>Stock</v>
       </c>
       <c r="B25" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="C25" t="str">
         <v/>
@@ -1609,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="F25" t="str">
-        <v>2.722</v>
+        <v>2.764</v>
       </c>
     </row>
     <row r="26">
@@ -1617,7 +1771,7 @@
         <v>Stock</v>
       </c>
       <c r="B26" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="C26" t="str">
         <v/>
@@ -1626,10 +1780,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E26" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" t="str">
-        <v>3.050</v>
+        <v>5.909</v>
       </c>
     </row>
     <row r="27">
@@ -1637,7 +1791,7 @@
         <v>Stock</v>
       </c>
       <c r="B27" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="C27" t="str">
         <v/>
@@ -1646,10 +1800,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E27" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F27" t="str">
-        <v>5.229</v>
+        <v>9.486</v>
       </c>
     </row>
     <row r="28">
@@ -1657,7 +1811,7 @@
         <v>Stock</v>
       </c>
       <c r="B28" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="C28" t="str">
         <v/>
@@ -1669,7 +1823,7 @@
         <v>1</v>
       </c>
       <c r="F28" t="str">
-        <v>2.639</v>
+        <v>2.252</v>
       </c>
     </row>
     <row r="29">
@@ -1677,7 +1831,7 @@
         <v>Stock</v>
       </c>
       <c r="B29" t="str">
-        <v>MORA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="C29" t="str">
         <v/>
@@ -1689,7 +1843,7 @@
         <v>1</v>
       </c>
       <c r="F29" t="str">
-        <v>2.411</v>
+        <v>2.291</v>
       </c>
     </row>
     <row r="30">
@@ -1697,7 +1851,7 @@
         <v>Stock</v>
       </c>
       <c r="B30" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="C30" t="str">
         <v/>
@@ -1706,10 +1860,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E30" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="str">
-        <v>9.065</v>
+        <v>5.239</v>
       </c>
     </row>
     <row r="31">
@@ -1717,7 +1871,7 @@
         <v>Stock</v>
       </c>
       <c r="B31" t="str">
-        <v>NOCCIOLA</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="C31" t="str">
         <v/>
@@ -1726,10 +1880,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E31" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F31" t="str">
-        <v>8.812</v>
+        <v>2.609</v>
       </c>
     </row>
     <row r="32">
@@ -1737,7 +1891,7 @@
         <v>Stock</v>
       </c>
       <c r="B32" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>LIMONE</v>
       </c>
       <c r="C32" t="str">
         <v/>
@@ -1746,10 +1900,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E32" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F32" t="str">
-        <v>2.652</v>
+        <v>10.105</v>
       </c>
     </row>
     <row r="33">
@@ -1757,7 +1911,7 @@
         <v>Stock</v>
       </c>
       <c r="B33" t="str">
-        <v>PASSION FRUIT</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="C33" t="str">
         <v/>
@@ -1766,10 +1920,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E33" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" t="str">
-        <v>4.986</v>
+        <v>2.752</v>
       </c>
     </row>
     <row r="34">
@@ -1777,7 +1931,7 @@
         <v>Stock</v>
       </c>
       <c r="B34" t="str">
-        <v>PERA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="C34" t="str">
         <v/>
@@ -1789,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="F34" t="str">
-        <v>2.160</v>
+        <v>2.846</v>
       </c>
     </row>
     <row r="35">
@@ -1797,7 +1951,7 @@
         <v>Stock</v>
       </c>
       <c r="B35" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="C35" t="str">
         <v/>
@@ -1809,7 +1963,7 @@
         <v>1</v>
       </c>
       <c r="F35" t="str">
-        <v>2.917</v>
+        <v>2.722</v>
       </c>
     </row>
     <row r="36">
@@ -1817,7 +1971,7 @@
         <v>Stock</v>
       </c>
       <c r="B36" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="C36" t="str">
         <v/>
@@ -1829,7 +1983,7 @@
         <v>1</v>
       </c>
       <c r="F36" t="str">
-        <v>2.841</v>
+        <v>3.050</v>
       </c>
     </row>
     <row r="37">
@@ -1837,7 +1991,7 @@
         <v>Stock</v>
       </c>
       <c r="B37" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="C37" t="str">
         <v/>
@@ -1846,10 +2000,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E37" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" t="str">
-        <v>2.806</v>
+        <v>5.229</v>
       </c>
     </row>
     <row r="38">
@@ -1857,7 +2011,7 @@
         <v>Stock</v>
       </c>
       <c r="B38" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="C38" t="str">
         <v/>
@@ -1869,7 +2023,7 @@
         <v>1</v>
       </c>
       <c r="F38" t="str">
-        <v>3.101</v>
+        <v>2.639</v>
       </c>
     </row>
     <row r="39">
@@ -1877,7 +2031,7 @@
         <v>Stock</v>
       </c>
       <c r="B39" t="str">
-        <v>STRACCIATELLA</v>
+        <v>MORA</v>
       </c>
       <c r="C39" t="str">
         <v/>
@@ -1886,10 +2040,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E39" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F39" t="str">
-        <v>8.617</v>
+        <v>2.411</v>
       </c>
     </row>
     <row r="40">
@@ -1897,7 +2051,7 @@
         <v>Stock</v>
       </c>
       <c r="B40" t="str">
-        <v>TIRAMISU'</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="C40" t="str">
         <v/>
@@ -1906,10 +2060,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E40" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40" t="str">
-        <v>5.277</v>
+        <v>9.065</v>
       </c>
     </row>
     <row r="41">
@@ -1917,7 +2071,7 @@
         <v>Stock</v>
       </c>
       <c r="B41" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="C41" t="str">
         <v/>
@@ -1926,10 +2080,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E41" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F41" t="str">
-        <v>3.055</v>
+        <v>11.651</v>
       </c>
     </row>
     <row r="42">
@@ -1937,7 +2091,7 @@
         <v>Stock</v>
       </c>
       <c r="B42" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="C42" t="str">
         <v/>
@@ -1949,7 +2103,7 @@
         <v>1</v>
       </c>
       <c r="F42" t="str">
-        <v>3.029</v>
+        <v>2.652</v>
       </c>
     </row>
     <row r="43">
@@ -1957,7 +2111,7 @@
         <v>Stock</v>
       </c>
       <c r="B43" t="str">
-        <v>PENSIERO</v>
+        <v>PAPAYA</v>
       </c>
       <c r="C43" t="str">
         <v/>
@@ -1969,7 +2123,7 @@
         <v>1</v>
       </c>
       <c r="F43" t="str">
-        <v>2.916</v>
+        <v>2.624</v>
       </c>
     </row>
     <row r="44">
@@ -1977,7 +2131,7 @@
         <v>Stock</v>
       </c>
       <c r="B44" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="C44" t="str">
         <v/>
@@ -1989,7 +2143,7 @@
         <v>2</v>
       </c>
       <c r="F44" t="str">
-        <v>5.346</v>
+        <v>4.986</v>
       </c>
     </row>
     <row r="45">
@@ -1997,7 +2151,7 @@
         <v>Stock</v>
       </c>
       <c r="B45" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="C45" t="str">
         <v/>
@@ -2009,7 +2163,7 @@
         <v>1</v>
       </c>
       <c r="F45" t="str">
-        <v>2.732</v>
+        <v>2.917</v>
       </c>
     </row>
     <row r="46">
@@ -2017,7 +2171,7 @@
         <v>Stock</v>
       </c>
       <c r="B46" t="str">
-        <v>MONT BLANC</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="C46" t="str">
         <v/>
@@ -2026,10 +2180,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E46" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" t="str">
-        <v>3.300</v>
+        <v>5.406</v>
       </c>
     </row>
     <row r="47">
@@ -2037,7 +2191,7 @@
         <v>Stock</v>
       </c>
       <c r="B47" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>POLLICINA</v>
       </c>
       <c r="C47" t="str">
         <v/>
@@ -2049,7 +2203,7 @@
         <v>1</v>
       </c>
       <c r="F47" t="str">
-        <v>3.287</v>
+        <v>2.736</v>
       </c>
     </row>
     <row r="48">
@@ -2057,7 +2211,7 @@
         <v>Stock</v>
       </c>
       <c r="B48" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="C48" t="str">
         <v/>
@@ -2069,7 +2223,7 @@
         <v>1</v>
       </c>
       <c r="F48" t="str">
-        <v>2.807</v>
+        <v>2.806</v>
       </c>
     </row>
     <row r="49">
@@ -2077,7 +2231,7 @@
         <v>Stock</v>
       </c>
       <c r="B49" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="C49" t="str">
         <v/>
@@ -2089,7 +2243,7 @@
         <v>1</v>
       </c>
       <c r="F49" t="str">
-        <v>2.827</v>
+        <v>3.101</v>
       </c>
     </row>
     <row r="50">
@@ -2097,7 +2251,7 @@
         <v>Stock</v>
       </c>
       <c r="B50" t="str">
-        <v>SACHER TORTE</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="C50" t="str">
         <v/>
@@ -2106,10 +2260,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E50" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50" t="str">
-        <v>2.746</v>
+        <v>5.744</v>
       </c>
     </row>
     <row r="51">
@@ -2117,7 +2271,7 @@
         <v>Stock</v>
       </c>
       <c r="B51" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="C51" t="str">
         <v/>
@@ -2126,10 +2280,10 @@
         <v>Mantenimento</v>
       </c>
       <c r="E51" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F51" t="str">
-        <v>3.169</v>
+        <v>5.277</v>
       </c>
     </row>
     <row r="52">
@@ -2137,7 +2291,7 @@
         <v>Stock</v>
       </c>
       <c r="B52" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="C52" t="str">
         <v/>
@@ -2149,19 +2303,239 @@
         <v>1</v>
       </c>
       <c r="F52" t="str">
-        <v>2.586</v>
+        <v>2.090</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B53" t="str">
+        <v>CIOCCOLATO WASABI</v>
+      </c>
+      <c r="C53" t="str">
+        <v/>
+      </c>
+      <c r="D53" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E53" t="str">
+        <v>1</v>
+      </c>
+      <c r="F53" t="str">
+        <v>3.055</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B54" t="str">
+        <v>ZABAIONE GELATO</v>
+      </c>
+      <c r="C54" t="str">
+        <v/>
+      </c>
+      <c r="D54" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E54" t="str">
+        <v>1</v>
+      </c>
+      <c r="F54" t="str">
+        <v>3.029</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B55" t="str">
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+      </c>
+      <c r="C55" t="str">
+        <v/>
+      </c>
+      <c r="D55" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E55" t="str">
+        <v>2</v>
+      </c>
+      <c r="F55" t="str">
+        <v>5.502</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B56" t="str">
+        <v>TE VERDE MATCHA</v>
+      </c>
+      <c r="C56" t="str">
+        <v/>
+      </c>
+      <c r="D56" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E56" t="str">
+        <v>2</v>
+      </c>
+      <c r="F56" t="str">
+        <v>5.346</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B57" t="str">
+        <v>PISTACCHIO SIRIANO</v>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E57" t="str">
+        <v>3</v>
+      </c>
+      <c r="F57" t="str">
+        <v>8.566</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B58" t="str">
+        <v>AVOCADO LIME E VINO BIANCO</v>
+      </c>
+      <c r="C58" t="str">
+        <v/>
+      </c>
+      <c r="D58" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E58" t="str">
+        <v>1</v>
+      </c>
+      <c r="F58" t="str">
+        <v>3.108</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B59" t="str">
+        <v>ZABAIONE AL SAKE'</v>
+      </c>
+      <c r="C59" t="str">
+        <v/>
+      </c>
+      <c r="D59" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E59" t="str">
+        <v>1</v>
+      </c>
+      <c r="F59" t="str">
+        <v>3.287</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B60" t="str">
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+      </c>
+      <c r="C60" t="str">
+        <v/>
+      </c>
+      <c r="D60" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E60" t="str">
+        <v>1</v>
+      </c>
+      <c r="F60" t="str">
+        <v>2.807</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B61" t="str">
+        <v>SACHER TORTE</v>
+      </c>
+      <c r="C61" t="str">
+        <v/>
+      </c>
+      <c r="D61" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E61" t="str">
+        <v>1</v>
+      </c>
+      <c r="F61" t="str">
+        <v>2.746</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B62" t="str">
+        <v>CASTAGNA AL WHISKY</v>
+      </c>
+      <c r="C62" t="str">
+        <v/>
+      </c>
+      <c r="D62" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E62" t="str">
+        <v>1</v>
+      </c>
+      <c r="F62" t="str">
+        <v>3.169</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Stock</v>
+      </c>
+      <c r="B63" t="str">
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+      </c>
+      <c r="C63" t="str">
+        <v/>
+      </c>
+      <c r="D63" t="str">
+        <v>Mantenimento</v>
+      </c>
+      <c r="E63" t="str">
+        <v>1</v>
+      </c>
+      <c r="F63" t="str">
+        <v>2.965</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F63"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2257,10 +2631,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E5" t="str">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" t="str">
-        <v>20.534</v>
+        <v>17.642</v>
       </c>
     </row>
     <row r="6">
@@ -2268,7 +2642,7 @@
         <v>Stock</v>
       </c>
       <c r="B6" t="str">
-        <v>BANANA E LIME</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -2280,7 +2654,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="str">
-        <v>2.353</v>
+        <v>2.820</v>
       </c>
     </row>
     <row r="7">
@@ -2288,7 +2662,7 @@
         <v>Stock</v>
       </c>
       <c r="B7" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="C7" t="str">
         <v/>
@@ -2300,7 +2674,7 @@
         <v>2</v>
       </c>
       <c r="F7" t="str">
-        <v>5.470</v>
+        <v>5.905</v>
       </c>
     </row>
     <row r="8">
@@ -2308,7 +2682,7 @@
         <v>Stock</v>
       </c>
       <c r="B8" t="str">
-        <v>BIANCANEVE</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -2320,7 +2694,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="str">
-        <v>2.822</v>
+        <v>2.542</v>
       </c>
     </row>
     <row r="9">
@@ -2328,7 +2702,7 @@
         <v>Stock</v>
       </c>
       <c r="B9" t="str">
-        <v>CAFFE'</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="C9" t="str">
         <v/>
@@ -2337,10 +2711,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E9" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" t="str">
-        <v>2.565</v>
+        <v>6.333</v>
       </c>
     </row>
     <row r="10">
@@ -2348,7 +2722,7 @@
         <v>Stock</v>
       </c>
       <c r="B10" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="C10" t="str">
         <v/>
@@ -2357,10 +2731,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E10" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="str">
-        <v>5.110</v>
+        <v>3.185</v>
       </c>
     </row>
     <row r="11">
@@ -2368,7 +2742,7 @@
         <v>Stock</v>
       </c>
       <c r="B11" t="str">
-        <v>CIOCCOLATO</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="C11" t="str">
         <v/>
@@ -2380,7 +2754,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="str">
-        <v>3.092</v>
+        <v>2.989</v>
       </c>
     </row>
     <row r="12">
@@ -2388,7 +2762,7 @@
         <v>Stock</v>
       </c>
       <c r="B12" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="C12" t="str">
         <v/>
@@ -2400,7 +2774,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="str">
-        <v>3.185</v>
+        <v>3.222</v>
       </c>
     </row>
     <row r="13">
@@ -2408,7 +2782,7 @@
         <v>Stock</v>
       </c>
       <c r="B13" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="C13" t="str">
         <v/>
@@ -2420,7 +2794,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="str">
-        <v>2.989</v>
+        <v>2.940</v>
       </c>
     </row>
     <row r="14">
@@ -2428,7 +2802,7 @@
         <v>Stock</v>
       </c>
       <c r="B14" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="C14" t="str">
         <v/>
@@ -2437,10 +2811,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E14" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" t="str">
-        <v>2.752</v>
+        <v>5.880</v>
       </c>
     </row>
     <row r="15">
@@ -2448,7 +2822,7 @@
         <v>Stock</v>
       </c>
       <c r="B15" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -2460,7 +2834,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="str">
-        <v>3.222</v>
+        <v>3.113</v>
       </c>
     </row>
     <row r="16">
@@ -2468,7 +2842,7 @@
         <v>Stock</v>
       </c>
       <c r="B16" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="C16" t="str">
         <v/>
@@ -2480,7 +2854,7 @@
         <v>2</v>
       </c>
       <c r="F16" t="str">
-        <v>5.999</v>
+        <v>5.172</v>
       </c>
     </row>
     <row r="17">
@@ -2488,7 +2862,7 @@
         <v>Stock</v>
       </c>
       <c r="B17" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="C17" t="str">
         <v/>
@@ -2497,10 +2871,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E17" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="str">
-        <v>5.880</v>
+        <v>7.689</v>
       </c>
     </row>
     <row r="18">
@@ -2508,7 +2882,7 @@
         <v>Stock</v>
       </c>
       <c r="B18" t="str">
-        <v>COCCO CREMA</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="C18" t="str">
         <v/>
@@ -2520,7 +2894,7 @@
         <v>2</v>
       </c>
       <c r="F18" t="str">
-        <v>5.879</v>
+        <v>5.020</v>
       </c>
     </row>
     <row r="19">
@@ -2528,7 +2902,7 @@
         <v>Stock</v>
       </c>
       <c r="B19" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="C19" t="str">
         <v/>
@@ -2537,10 +2911,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E19" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="str">
-        <v>5.330</v>
+        <v>2.705</v>
       </c>
     </row>
     <row r="20">
@@ -2548,7 +2922,7 @@
         <v>Stock</v>
       </c>
       <c r="B20" t="str">
-        <v>CREMA AGNESE</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="C20" t="str">
         <v/>
@@ -2557,10 +2931,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E20" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="str">
-        <v>7.833</v>
+        <v>5.607</v>
       </c>
     </row>
     <row r="21">
@@ -2568,7 +2942,7 @@
         <v>Stock</v>
       </c>
       <c r="B21" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="C21" t="str">
         <v/>
@@ -2577,10 +2951,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E21" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" t="str">
-        <v>2.403</v>
+        <v>4.747</v>
       </c>
     </row>
     <row r="22">
@@ -2588,7 +2962,7 @@
         <v>Stock</v>
       </c>
       <c r="B22" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="C22" t="str">
         <v/>
@@ -2597,10 +2971,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E22" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" t="str">
-        <v>2.705</v>
+        <v>4.756</v>
       </c>
     </row>
     <row r="23">
@@ -2608,7 +2982,7 @@
         <v>Stock</v>
       </c>
       <c r="B23" t="str">
-        <v>FIORDILATTE</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="C23" t="str">
         <v/>
@@ -2617,10 +2991,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E23" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="str">
-        <v>5.607</v>
+        <v>2.276</v>
       </c>
     </row>
     <row r="24">
@@ -2628,7 +3002,7 @@
         <v>Stock</v>
       </c>
       <c r="B24" t="str">
-        <v>FRAGOLA</v>
+        <v>LIMONE</v>
       </c>
       <c r="C24" t="str">
         <v/>
@@ -2637,10 +3011,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E24" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="str">
-        <v>7.213</v>
+        <v>4.937</v>
       </c>
     </row>
     <row r="25">
@@ -2648,7 +3022,7 @@
         <v>Stock</v>
       </c>
       <c r="B25" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="C25" t="str">
         <v/>
@@ -2657,10 +3031,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E25" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" t="str">
-        <v>4.756</v>
+        <v>2.838</v>
       </c>
     </row>
     <row r="26">
@@ -2668,7 +3042,7 @@
         <v>Stock</v>
       </c>
       <c r="B26" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="C26" t="str">
         <v/>
@@ -2680,7 +3054,7 @@
         <v>1</v>
       </c>
       <c r="F26" t="str">
-        <v>2.276</v>
+        <v>2.935</v>
       </c>
     </row>
     <row r="27">
@@ -2688,7 +3062,7 @@
         <v>Stock</v>
       </c>
       <c r="B27" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="C27" t="str">
         <v/>
@@ -2700,7 +3074,7 @@
         <v>1</v>
       </c>
       <c r="F27" t="str">
-        <v>2.659</v>
+        <v>2.238</v>
       </c>
     </row>
     <row r="28">
@@ -2708,7 +3082,7 @@
         <v>Stock</v>
       </c>
       <c r="B28" t="str">
-        <v>LIMONE</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="C28" t="str">
         <v/>
@@ -2717,10 +3091,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E28" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" t="str">
-        <v>4.937</v>
+        <v>2.427</v>
       </c>
     </row>
     <row r="29">
@@ -2728,7 +3102,7 @@
         <v>Stock</v>
       </c>
       <c r="B29" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="C29" t="str">
         <v/>
@@ -2740,7 +3114,7 @@
         <v>2</v>
       </c>
       <c r="F29" t="str">
-        <v>5.557</v>
+        <v>5.760</v>
       </c>
     </row>
     <row r="30">
@@ -2748,7 +3122,7 @@
         <v>Stock</v>
       </c>
       <c r="B30" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="C30" t="str">
         <v/>
@@ -2760,7 +3134,7 @@
         <v>1</v>
       </c>
       <c r="F30" t="str">
-        <v>2.935</v>
+        <v>2.977</v>
       </c>
     </row>
     <row r="31">
@@ -2768,7 +3142,7 @@
         <v>Stock</v>
       </c>
       <c r="B31" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>PERA</v>
       </c>
       <c r="C31" t="str">
         <v/>
@@ -2780,7 +3154,7 @@
         <v>1</v>
       </c>
       <c r="F31" t="str">
-        <v>2.378</v>
+        <v>2.377</v>
       </c>
     </row>
     <row r="32">
@@ -2788,7 +3162,7 @@
         <v>Stock</v>
       </c>
       <c r="B32" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="C32" t="str">
         <v/>
@@ -2797,10 +3171,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E32" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" t="str">
-        <v>4.634</v>
+        <v>2.493</v>
       </c>
     </row>
     <row r="33">
@@ -2808,7 +3182,7 @@
         <v>Stock</v>
       </c>
       <c r="B33" t="str">
-        <v>MIRTILLO</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="C33" t="str">
         <v/>
@@ -2817,10 +3191,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E33" t="str">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F33" t="str">
-        <v>2.427</v>
+        <v>19.767</v>
       </c>
     </row>
     <row r="34">
@@ -2828,7 +3202,7 @@
         <v>Stock</v>
       </c>
       <c r="B34" t="str">
-        <v>NOCCIOLA</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="C34" t="str">
         <v/>
@@ -2837,10 +3211,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E34" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="str">
-        <v>5.610</v>
+        <v>3.139</v>
       </c>
     </row>
     <row r="35">
@@ -2848,7 +3222,7 @@
         <v>Stock</v>
       </c>
       <c r="B35" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>SEADAS</v>
       </c>
       <c r="C35" t="str">
         <v/>
@@ -2860,7 +3234,7 @@
         <v>1</v>
       </c>
       <c r="F35" t="str">
-        <v>2.977</v>
+        <v>2.879</v>
       </c>
     </row>
     <row r="36">
@@ -2868,7 +3242,7 @@
         <v>Stock</v>
       </c>
       <c r="B36" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="C36" t="str">
         <v/>
@@ -2877,10 +3251,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E36" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F36" t="str">
-        <v>2.392</v>
+        <v>13.858</v>
       </c>
     </row>
     <row r="37">
@@ -2888,7 +3262,7 @@
         <v>Stock</v>
       </c>
       <c r="B37" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>YOGURT</v>
       </c>
       <c r="C37" t="str">
         <v/>
@@ -2897,10 +3271,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E37" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" t="str">
-        <v>2.493</v>
+        <v>5.688</v>
       </c>
     </row>
     <row r="38">
@@ -2908,7 +3282,7 @@
         <v>Stock</v>
       </c>
       <c r="B38" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="C38" t="str">
         <v/>
@@ -2917,10 +3291,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E38" t="str">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F38" t="str">
-        <v>21.856</v>
+        <v>2.837</v>
       </c>
     </row>
     <row r="39">
@@ -2928,7 +3302,7 @@
         <v>Stock</v>
       </c>
       <c r="B39" t="str">
-        <v>POLLICINA</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="C39" t="str">
         <v/>
@@ -2940,7 +3314,7 @@
         <v>1</v>
       </c>
       <c r="F39" t="str">
-        <v>3.137</v>
+        <v>3.107</v>
       </c>
     </row>
     <row r="40">
@@ -2948,7 +3322,7 @@
         <v>Stock</v>
       </c>
       <c r="B40" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="C40" t="str">
         <v/>
@@ -2957,10 +3331,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E40" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" t="str">
-        <v>3.139</v>
+        <v>5.376</v>
       </c>
     </row>
     <row r="41">
@@ -2968,7 +3342,7 @@
         <v>Stock</v>
       </c>
       <c r="B41" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="C41" t="str">
         <v/>
@@ -2980,7 +3354,7 @@
         <v>1</v>
       </c>
       <c r="F41" t="str">
-        <v>2.809</v>
+        <v>2.521</v>
       </c>
     </row>
     <row r="42">
@@ -2988,7 +3362,7 @@
         <v>Stock</v>
       </c>
       <c r="B42" t="str">
-        <v>SEADAS</v>
+        <v>SEMIFREDDO  TIRAMISU</v>
       </c>
       <c r="C42" t="str">
         <v/>
@@ -3000,7 +3374,7 @@
         <v>1</v>
       </c>
       <c r="F42" t="str">
-        <v>2.879</v>
+        <v>750</v>
       </c>
     </row>
     <row r="43">
@@ -3008,7 +3382,7 @@
         <v>Stock</v>
       </c>
       <c r="B43" t="str">
-        <v>STRACCIATELLA</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="C43" t="str">
         <v/>
@@ -3017,10 +3391,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E43" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F43" t="str">
-        <v>16.658</v>
+        <v>3.327</v>
       </c>
     </row>
     <row r="44">
@@ -3028,7 +3402,7 @@
         <v>Stock</v>
       </c>
       <c r="B44" t="str">
-        <v>YOGURT</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="C44" t="str">
         <v/>
@@ -3040,7 +3414,7 @@
         <v>1</v>
       </c>
       <c r="F44" t="str">
-        <v>2.927</v>
+        <v>1.001</v>
       </c>
     </row>
     <row r="45">
@@ -3048,7 +3422,7 @@
         <v>Stock</v>
       </c>
       <c r="B45" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="C45" t="str">
         <v/>
@@ -3057,10 +3431,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E45" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F45" t="str">
-        <v>3.052</v>
+        <v>6.708</v>
       </c>
     </row>
     <row r="46">
@@ -3068,7 +3442,7 @@
         <v>Stock</v>
       </c>
       <c r="B46" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="C46" t="str">
         <v/>
@@ -3080,7 +3454,7 @@
         <v>1</v>
       </c>
       <c r="F46" t="str">
-        <v>2.837</v>
+        <v>2.675</v>
       </c>
     </row>
     <row r="47">
@@ -3088,7 +3462,7 @@
         <v>Stock</v>
       </c>
       <c r="B47" t="str">
-        <v>SACRIPANTE</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="C47" t="str">
         <v/>
@@ -3097,10 +3471,10 @@
         <v>Esaurito</v>
       </c>
       <c r="E47" t="str">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F47" t="str">
-        <v>3.107</v>
+        <v>3.717</v>
       </c>
     </row>
     <row r="48">
@@ -3108,7 +3482,7 @@
         <v>Stock</v>
       </c>
       <c r="B48" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="C48" t="str">
         <v/>
@@ -3117,162 +3491,22 @@
         <v>Esaurito</v>
       </c>
       <c r="E48" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="str">
-        <v>8.065</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>Stock</v>
-      </c>
-      <c r="B49" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
-      </c>
-      <c r="C49" t="str">
-        <v/>
-      </c>
-      <c r="D49" t="str">
-        <v>Esaurito</v>
-      </c>
-      <c r="E49" t="str">
-        <v>1</v>
-      </c>
-      <c r="F49" t="str">
-        <v>1.017</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>Stock</v>
-      </c>
-      <c r="B50" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
-      </c>
-      <c r="C50" t="str">
-        <v/>
-      </c>
-      <c r="D50" t="str">
-        <v>Esaurito</v>
-      </c>
-      <c r="E50" t="str">
-        <v>1</v>
-      </c>
-      <c r="F50" t="str">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>Stock</v>
-      </c>
-      <c r="B51" t="str">
-        <v>MONT BLANC</v>
-      </c>
-      <c r="C51" t="str">
-        <v/>
-      </c>
-      <c r="D51" t="str">
-        <v>Esaurito</v>
-      </c>
-      <c r="E51" t="str">
-        <v>1</v>
-      </c>
-      <c r="F51" t="str">
-        <v>3.053</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>Stock</v>
-      </c>
-      <c r="B52" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
-      </c>
-      <c r="C52" t="str">
-        <v/>
-      </c>
-      <c r="D52" t="str">
-        <v>Esaurito</v>
-      </c>
-      <c r="E52" t="str">
-        <v>1</v>
-      </c>
-      <c r="F52" t="str">
-        <v>3.275</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>Stock</v>
-      </c>
-      <c r="B53" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
-      </c>
-      <c r="C53" t="str">
-        <v/>
-      </c>
-      <c r="D53" t="str">
-        <v>Esaurito</v>
-      </c>
-      <c r="E53" t="str">
-        <v>1</v>
-      </c>
-      <c r="F53" t="str">
-        <v>2.675</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>Stock</v>
-      </c>
-      <c r="B54" t="str">
-        <v>CREMA MASCARPONE</v>
-      </c>
-      <c r="C54" t="str">
-        <v/>
-      </c>
-      <c r="D54" t="str">
-        <v>Esaurito</v>
-      </c>
-      <c r="E54" t="str">
-        <v>5</v>
-      </c>
-      <c r="F54" t="str">
-        <v>2.670</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>Stock</v>
-      </c>
-      <c r="B55" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
-      </c>
-      <c r="C55" t="str">
-        <v/>
-      </c>
-      <c r="D55" t="str">
-        <v>Esaurito</v>
-      </c>
-      <c r="E55" t="str">
-        <v>2</v>
-      </c>
-      <c r="F55" t="str">
         <v>5.842</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F48"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C82"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3309,29 +3543,29 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C4" t="str">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BANANA E LIME</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>CACHI</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
@@ -3342,7 +3576,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>CIOCCOLATO</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B7" t="str">
         <v>Da Ordinare</v>
@@ -3353,7 +3587,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
@@ -3364,7 +3598,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
@@ -3375,117 +3609,117 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CACHI</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C10" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C12" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C14" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>COCCO CREMA</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C18" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -3496,18 +3730,18 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>FIORDILATTE</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C21" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>FRAGOLA</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
@@ -3518,18 +3752,18 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>LEMON CURD</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>LIMONE</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
@@ -3540,29 +3774,29 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
@@ -3573,7 +3807,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
@@ -3584,18 +3818,18 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MORA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
@@ -3606,7 +3840,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>NOCCIOLA</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
@@ -3617,18 +3851,18 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>LIMONE</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>PASSION FRUIT</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
@@ -3639,51 +3873,51 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>PERA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -3694,18 +3928,18 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>STRACCIATELLA</v>
+        <v>MORA</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>TIRAMISU'</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
@@ -3716,7 +3950,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -3727,18 +3961,18 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C42" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>PENSIERO</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
@@ -3749,7 +3983,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
@@ -3760,29 +3994,29 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>MONT BLANC</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
@@ -3793,40 +4027,40 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C48" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C49" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>SACHER TORTE</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C50" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
@@ -3837,128 +4071,128 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C52" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ALBICOCCA</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>BIANCANEVE</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>CAFFE'</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C57" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>CREMA AGNESE</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C60" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C61" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C62" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
@@ -3969,7 +4203,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
@@ -3980,18 +4214,18 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C65" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>MIRTILLO</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
@@ -4002,7 +4236,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
@@ -4013,18 +4247,18 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>POLLICINA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
@@ -4035,7 +4269,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>SEADAS</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
@@ -4046,7 +4280,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>YOGURT</v>
+        <v>PERA</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
@@ -4057,7 +4291,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
@@ -4068,7 +4302,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>SACRIPANTE</v>
+        <v>SEADAS</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
@@ -4079,18 +4313,18 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>YOGURT</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
@@ -4101,29 +4335,84 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>SEMIFREDDO  TIRAMISU</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>MONT BLANC</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C78" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>TORTA CAPRESE</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C79" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>EVERGREEN  BRONTE VEGAN</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C80" t="str">
         <v>3</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C81" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>CREMA MASCARPONE</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C82" t="str">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C82"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>